<commit_message>
flow and slope scaling
</commit_message>
<xml_diff>
--- a/slope_analysis/excel_algorithm.xlsx
+++ b/slope_analysis/excel_algorithm.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netafim-my.sharepoint.com/personal/avi_schweitzer_netafim_com/Documents/MyProjects/gravimetric_flow_sensor/grav_flow_sensor/slope_analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="66" documentId="8_{BAF58770-6495-4278-924C-B5EA990002C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC199D2A-7E47-4FBC-8F47-52714596AD2C}"/>
+  <xr:revisionPtr revIDLastSave="68" documentId="8_{BAF58770-6495-4278-924C-B5EA990002C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D216E34-635C-40DB-A852-50C0131484FF}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="38700" windowHeight="15225" xr2:uid="{17676617-7F34-427D-89E7-77851C69EA55}"/>
+    <workbookView xWindow="-28905" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{17676617-7F34-427D-89E7-77851C69EA55}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -4359,6 +4359,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -4677,131 +4681,131 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5F25604-130F-48A0-80B7-7455EADA05D8}">
   <dimension ref="A1:AF191"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="16" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="13" max="16" width="14.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>-1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>-10</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>-17</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>-9</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>-3</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>-5</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>4</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>3</v>
       </c>
@@ -4813,7 +4817,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>3</v>
       </c>
@@ -4825,7 +4829,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>4</v>
       </c>
@@ -4837,7 +4841,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>4</v>
       </c>
@@ -4849,7 +4853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>3</v>
       </c>
@@ -4861,7 +4865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>4</v>
       </c>
@@ -4873,7 +4877,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>3</v>
       </c>
@@ -4885,7 +4889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>0</v>
       </c>
@@ -4897,7 +4901,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>-12</v>
       </c>
@@ -4909,7 +4913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>-3</v>
       </c>
@@ -4921,7 +4925,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>0</v>
       </c>
@@ -4945,7 +4949,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>2</v>
       </c>
@@ -4971,7 +4975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>13</v>
       </c>
@@ -4997,7 +5001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>16</v>
       </c>
@@ -5023,7 +5027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>20</v>
       </c>
@@ -5049,7 +5053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>10</v>
       </c>
@@ -5075,7 +5079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>4</v>
       </c>
@@ -5101,7 +5105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>26</v>
       </c>
@@ -5127,7 +5131,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>32</v>
       </c>
@@ -5155,7 +5159,7 @@
       <c r="X41" s="5"/>
       <c r="Y41" s="5"/>
     </row>
-    <row r="42" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>36</v>
       </c>
@@ -5181,7 +5185,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>40</v>
       </c>
@@ -5207,7 +5211,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>43</v>
       </c>
@@ -5233,7 +5237,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>46</v>
       </c>
@@ -5259,7 +5263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>49</v>
       </c>
@@ -5319,7 +5323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>52</v>
       </c>
@@ -5386,7 +5390,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>55</v>
       </c>
@@ -5469,7 +5473,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="49" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>58</v>
       </c>
@@ -5558,7 +5562,7 @@
       <c r="AB49" s="6"/>
       <c r="AC49" s="6"/>
     </row>
-    <row r="50" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>60</v>
       </c>
@@ -5641,7 +5645,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="51" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>64</v>
       </c>
@@ -5724,7 +5728,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="52" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>68</v>
       </c>
@@ -5807,7 +5811,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="53" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>72</v>
       </c>
@@ -5874,7 +5878,7 @@
         <v>3.2857142857142856</v>
       </c>
       <c r="R53">
-        <f t="shared" si="9"/>
+        <f>Q53*360</f>
         <v>1182.8571428571429</v>
       </c>
       <c r="S53">
@@ -5890,7 +5894,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="54" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>75</v>
       </c>
@@ -5982,7 +5986,7 @@
       <c r="AE54" s="6"/>
       <c r="AF54" s="6"/>
     </row>
-    <row r="55" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>79</v>
       </c>
@@ -6065,7 +6069,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="56" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>82</v>
       </c>
@@ -6148,7 +6152,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="57" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>86</v>
       </c>
@@ -6231,7 +6235,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="58" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>88</v>
       </c>
@@ -6314,7 +6318,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="59" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>92</v>
       </c>
@@ -6397,7 +6401,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="60" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>97</v>
       </c>
@@ -6480,7 +6484,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="61" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>100</v>
       </c>
@@ -6563,7 +6567,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="62" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>101</v>
       </c>
@@ -6646,7 +6650,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="63" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>100</v>
       </c>
@@ -6729,7 +6733,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="64" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>105</v>
       </c>
@@ -6812,7 +6816,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="65" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>111</v>
       </c>
@@ -6895,7 +6899,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="66" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>113</v>
       </c>
@@ -6978,7 +6982,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="67" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>115</v>
       </c>
@@ -7061,7 +7065,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="68" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>119</v>
       </c>
@@ -7144,7 +7148,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="69" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>124</v>
       </c>
@@ -7227,7 +7231,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="70" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>125</v>
       </c>
@@ -7310,7 +7314,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="71" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>105</v>
       </c>
@@ -7393,7 +7397,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="72" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>111</v>
       </c>
@@ -7476,7 +7480,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="73" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>137</v>
       </c>
@@ -7559,7 +7563,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="74" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>140</v>
       </c>
@@ -7642,7 +7646,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="75" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>120</v>
       </c>
@@ -7725,7 +7729,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="76" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>106</v>
       </c>
@@ -7808,7 +7812,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="77" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>150</v>
       </c>
@@ -7891,7 +7895,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="78" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>156</v>
       </c>
@@ -7974,7 +7978,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="79" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>148</v>
       </c>
@@ -8057,7 +8061,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="80" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>112</v>
       </c>
@@ -8140,7 +8144,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="81" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>154</v>
       </c>
@@ -8223,7 +8227,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="82" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>165</v>
       </c>
@@ -8306,7 +8310,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="83" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>150</v>
       </c>
@@ -8389,7 +8393,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="84" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>155</v>
       </c>
@@ -8472,7 +8476,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="85" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>180</v>
       </c>
@@ -8555,7 +8559,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="86" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>174</v>
       </c>
@@ -8638,7 +8642,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="87" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>173</v>
       </c>
@@ -8721,7 +8725,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="88" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>166</v>
       </c>
@@ -8804,7 +8808,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="89" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>190</v>
       </c>
@@ -8887,7 +8891,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="90" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A90">
         <v>194</v>
       </c>
@@ -8970,7 +8974,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="91" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A91">
         <v>184</v>
       </c>
@@ -9053,7 +9057,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="92" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A92">
         <v>195</v>
       </c>
@@ -9136,7 +9140,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="93" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A93">
         <v>187</v>
       </c>
@@ -9219,7 +9223,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="94" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A94">
         <v>191</v>
       </c>
@@ -9302,7 +9306,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="95" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A95">
         <v>213</v>
       </c>
@@ -9385,7 +9389,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="96" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A96">
         <v>218</v>
       </c>
@@ -9468,7 +9472,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="97" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A97">
         <v>213</v>
       </c>
@@ -9551,7 +9555,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="98" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A98">
         <v>199</v>
       </c>
@@ -9634,7 +9638,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="99" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A99">
         <v>223</v>
       </c>
@@ -9717,7 +9721,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="100" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A100">
         <v>229</v>
       </c>
@@ -9800,7 +9804,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="101" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A101">
         <v>234</v>
       </c>
@@ -9883,7 +9887,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="102" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A102">
         <v>241</v>
       </c>
@@ -9966,7 +9970,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="103" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A103">
         <v>239</v>
       </c>
@@ -10049,7 +10053,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="104" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A104">
         <v>217</v>
       </c>
@@ -10132,7 +10136,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="105" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A105">
         <v>232</v>
       </c>
@@ -10215,7 +10219,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="106" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A106">
         <v>250</v>
       </c>
@@ -10298,7 +10302,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="107" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A107">
         <v>253</v>
       </c>
@@ -10381,7 +10385,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="108" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A108">
         <v>237</v>
       </c>
@@ -10464,7 +10468,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="109" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A109">
         <v>231</v>
       </c>
@@ -10547,7 +10551,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="110" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A110">
         <v>262</v>
       </c>
@@ -10630,7 +10634,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="111" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A111">
         <v>267</v>
       </c>
@@ -10713,7 +10717,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="112" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A112">
         <v>270</v>
       </c>
@@ -10796,7 +10800,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="113" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A113">
         <v>273</v>
       </c>
@@ -10879,7 +10883,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="114" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A114">
         <v>271</v>
       </c>
@@ -10962,7 +10966,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="115" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A115">
         <v>278</v>
       </c>
@@ -11045,7 +11049,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="116" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A116">
         <v>261</v>
       </c>
@@ -11128,7 +11132,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="117" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A117">
         <v>271</v>
       </c>
@@ -11211,7 +11215,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="118" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A118">
         <v>290</v>
       </c>
@@ -11294,7 +11298,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="119" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A119">
         <v>295</v>
       </c>
@@ -11377,7 +11381,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="120" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A120">
         <v>284</v>
       </c>
@@ -11460,7 +11464,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="121" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A121">
         <v>274</v>
       </c>
@@ -11543,7 +11547,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="122" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A122">
         <v>298</v>
       </c>
@@ -11626,7 +11630,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="123" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A123">
         <v>307</v>
       </c>
@@ -11709,7 +11713,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="124" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A124">
         <v>312</v>
       </c>
@@ -11792,7 +11796,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="125" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A125">
         <v>316</v>
       </c>
@@ -11875,7 +11879,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="126" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A126">
         <v>319</v>
       </c>
@@ -11958,7 +11962,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="127" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A127">
         <v>323</v>
       </c>
@@ -12041,7 +12045,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="128" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A128">
         <v>325</v>
       </c>
@@ -12124,7 +12128,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="129" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A129">
         <v>328</v>
       </c>
@@ -12207,7 +12211,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="130" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A130">
         <v>330</v>
       </c>
@@ -12290,7 +12294,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="131" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A131">
         <v>332</v>
       </c>
@@ -12373,7 +12377,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="132" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A132">
         <v>336</v>
       </c>
@@ -12456,7 +12460,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="133" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A133">
         <v>323</v>
       </c>
@@ -12539,7 +12543,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="134" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A134">
         <v>313</v>
       </c>
@@ -12622,7 +12626,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="135" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A135">
         <v>340</v>
       </c>
@@ -12705,7 +12709,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="136" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A136">
         <v>346</v>
       </c>
@@ -12788,7 +12792,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="137" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A137">
         <v>330</v>
       </c>
@@ -12871,7 +12875,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="138" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A138">
         <v>354</v>
       </c>
@@ -12954,7 +12958,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="139" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A139">
         <v>360</v>
       </c>
@@ -13037,7 +13041,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="140" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A140">
         <v>363</v>
       </c>
@@ -13120,7 +13124,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="141" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A141">
         <v>367</v>
       </c>
@@ -13203,7 +13207,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="142" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A142">
         <v>373</v>
       </c>
@@ -13286,7 +13290,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="143" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A143">
         <v>376</v>
       </c>
@@ -13369,7 +13373,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="144" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A144">
         <v>379</v>
       </c>
@@ -13452,7 +13456,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="145" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A145">
         <v>380</v>
       </c>
@@ -13535,7 +13539,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="146" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A146">
         <v>381</v>
       </c>
@@ -13618,7 +13622,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="147" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A147">
         <v>390</v>
       </c>
@@ -13701,7 +13705,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="148" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A148">
         <v>392</v>
       </c>
@@ -13784,7 +13788,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="149" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A149">
         <v>397</v>
       </c>
@@ -13867,7 +13871,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="150" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A150">
         <v>399</v>
       </c>
@@ -13950,7 +13954,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="151" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A151">
         <v>392</v>
       </c>
@@ -14033,7 +14037,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="152" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A152">
         <v>368</v>
       </c>
@@ -14116,7 +14120,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="153" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A153">
         <v>398</v>
       </c>
@@ -14199,7 +14203,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="154" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A154">
         <v>409</v>
       </c>
@@ -14282,7 +14286,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="155" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A155">
         <v>412</v>
       </c>
@@ -14365,7 +14369,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="156" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A156">
         <v>392</v>
       </c>
@@ -14448,7 +14452,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="157" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A157">
         <v>408</v>
       </c>
@@ -14531,7 +14535,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="158" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A158">
         <v>425</v>
       </c>
@@ -14614,7 +14618,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="159" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A159">
         <v>429</v>
       </c>
@@ -14697,7 +14701,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="160" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A160">
         <v>431</v>
       </c>
@@ -14760,7 +14764,7 @@
         <v>14073585</v>
       </c>
       <c r="Q160">
-        <f t="shared" si="44"/>
+        <f>M160/P160</f>
         <v>3.3612118021101232</v>
       </c>
       <c r="R160">
@@ -14780,7 +14784,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="161" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="161" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D161" s="4"/>
       <c r="E161" s="4"/>
       <c r="F161" s="4"/>
@@ -14795,7 +14799,7 @@
       <c r="O161" s="4"/>
       <c r="P161" s="4"/>
     </row>
-    <row r="162" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="162" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D162" s="4"/>
       <c r="E162" s="4"/>
       <c r="F162" s="4"/>
@@ -14810,7 +14814,7 @@
       <c r="O162" s="4"/>
       <c r="P162" s="4"/>
     </row>
-    <row r="163" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="163" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D163" s="4"/>
       <c r="E163" s="4"/>
       <c r="F163" s="4"/>
@@ -14825,7 +14829,7 @@
       <c r="O163" s="4"/>
       <c r="P163" s="4"/>
     </row>
-    <row r="164" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="164" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D164" s="4"/>
       <c r="E164" s="4"/>
       <c r="F164" s="4"/>
@@ -14840,7 +14844,7 @@
       <c r="O164" s="4"/>
       <c r="P164" s="4"/>
     </row>
-    <row r="165" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="165" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D165" s="4"/>
       <c r="E165" s="4"/>
       <c r="F165" s="4"/>
@@ -14855,7 +14859,7 @@
       <c r="O165" s="4"/>
       <c r="P165" s="4"/>
     </row>
-    <row r="166" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="166" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D166" s="4"/>
       <c r="E166" s="4"/>
       <c r="F166" s="4"/>
@@ -14870,7 +14874,7 @@
       <c r="O166" s="4"/>
       <c r="P166" s="4"/>
     </row>
-    <row r="167" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="167" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D167" s="4"/>
       <c r="E167" s="4"/>
       <c r="F167" s="4"/>
@@ -14885,7 +14889,7 @@
       <c r="O167" s="4"/>
       <c r="P167" s="4"/>
     </row>
-    <row r="168" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="168" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D168" s="4"/>
       <c r="E168" s="4"/>
       <c r="F168" s="4"/>
@@ -14900,7 +14904,7 @@
       <c r="O168" s="4"/>
       <c r="P168" s="4"/>
     </row>
-    <row r="169" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="169" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D169" s="4"/>
       <c r="E169" s="4"/>
       <c r="F169" s="4"/>
@@ -14915,7 +14919,7 @@
       <c r="O169" s="4"/>
       <c r="P169" s="4"/>
     </row>
-    <row r="170" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="170" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D170" s="4"/>
       <c r="E170" s="4"/>
       <c r="F170" s="4"/>
@@ -14930,7 +14934,7 @@
       <c r="O170" s="4"/>
       <c r="P170" s="4"/>
     </row>
-    <row r="171" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="171" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D171" s="4"/>
       <c r="E171" s="4"/>
       <c r="F171" s="4"/>
@@ -14945,7 +14949,7 @@
       <c r="O171" s="4"/>
       <c r="P171" s="4"/>
     </row>
-    <row r="172" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="172" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D172" s="4"/>
       <c r="E172" s="4"/>
       <c r="F172" s="4"/>
@@ -14960,7 +14964,7 @@
       <c r="O172" s="4"/>
       <c r="P172" s="4"/>
     </row>
-    <row r="173" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="173" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D173" s="4"/>
       <c r="E173" s="4"/>
       <c r="F173" s="4"/>
@@ -14975,7 +14979,7 @@
       <c r="O173" s="4"/>
       <c r="P173" s="4"/>
     </row>
-    <row r="174" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="174" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D174" s="4"/>
       <c r="E174" s="4"/>
       <c r="F174" s="4"/>
@@ -14990,7 +14994,7 @@
       <c r="O174" s="4"/>
       <c r="P174" s="4"/>
     </row>
-    <row r="175" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="175" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D175" s="4"/>
       <c r="E175" s="4"/>
       <c r="F175" s="4"/>
@@ -15005,7 +15009,7 @@
       <c r="O175" s="4"/>
       <c r="P175" s="4"/>
     </row>
-    <row r="176" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="176" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D176" s="4"/>
       <c r="E176" s="4"/>
       <c r="F176" s="4"/>
@@ -15020,7 +15024,7 @@
       <c r="O176" s="4"/>
       <c r="P176" s="4"/>
     </row>
-    <row r="177" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="177" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D177" s="4"/>
       <c r="E177" s="4"/>
       <c r="F177" s="4"/>
@@ -15035,7 +15039,7 @@
       <c r="O177" s="4"/>
       <c r="P177" s="4"/>
     </row>
-    <row r="178" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="178" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D178" s="4"/>
       <c r="E178" s="4"/>
       <c r="F178" s="4"/>
@@ -15050,7 +15054,7 @@
       <c r="O178" s="4"/>
       <c r="P178" s="4"/>
     </row>
-    <row r="179" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="179" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D179" s="4"/>
       <c r="E179" s="4"/>
       <c r="F179" s="4"/>
@@ -15065,7 +15069,7 @@
       <c r="O179" s="4"/>
       <c r="P179" s="4"/>
     </row>
-    <row r="180" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="180" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D180" s="4"/>
       <c r="E180" s="4"/>
       <c r="F180" s="4"/>
@@ -15080,7 +15084,7 @@
       <c r="O180" s="4"/>
       <c r="P180" s="4"/>
     </row>
-    <row r="181" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="181" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D181" s="4"/>
       <c r="E181" s="4"/>
       <c r="F181" s="4"/>
@@ -15095,7 +15099,7 @@
       <c r="O181" s="4"/>
       <c r="P181" s="4"/>
     </row>
-    <row r="182" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="182" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D182" s="4"/>
       <c r="E182" s="4"/>
       <c r="F182" s="4"/>
@@ -15110,7 +15114,7 @@
       <c r="O182" s="4"/>
       <c r="P182" s="4"/>
     </row>
-    <row r="183" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="183" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D183" s="4"/>
       <c r="E183" s="4"/>
       <c r="F183" s="4"/>
@@ -15125,7 +15129,7 @@
       <c r="O183" s="4"/>
       <c r="P183" s="4"/>
     </row>
-    <row r="184" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="184" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D184" s="4"/>
       <c r="E184" s="4"/>
       <c r="F184" s="4"/>
@@ -15140,7 +15144,7 @@
       <c r="O184" s="4"/>
       <c r="P184" s="4"/>
     </row>
-    <row r="185" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="185" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D185" s="4"/>
       <c r="E185" s="4"/>
       <c r="F185" s="4"/>
@@ -15155,7 +15159,7 @@
       <c r="O185" s="4"/>
       <c r="P185" s="4"/>
     </row>
-    <row r="186" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="186" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D186" s="4"/>
       <c r="E186" s="4"/>
       <c r="F186" s="4"/>
@@ -15170,7 +15174,7 @@
       <c r="O186" s="4"/>
       <c r="P186" s="4"/>
     </row>
-    <row r="187" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="187" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D187" s="4"/>
       <c r="E187" s="4"/>
       <c r="F187" s="4"/>
@@ -15185,7 +15189,7 @@
       <c r="O187" s="4"/>
       <c r="P187" s="4"/>
     </row>
-    <row r="188" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="188" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D188" s="4"/>
       <c r="E188" s="4"/>
       <c r="F188" s="4"/>
@@ -15200,7 +15204,7 @@
       <c r="O188" s="4"/>
       <c r="P188" s="4"/>
     </row>
-    <row r="189" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="189" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D189" s="4"/>
       <c r="E189" s="4"/>
       <c r="F189" s="4"/>
@@ -15215,7 +15219,7 @@
       <c r="O189" s="4"/>
       <c r="P189" s="4"/>
     </row>
-    <row r="190" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="190" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D190" s="4"/>
       <c r="E190" s="4"/>
       <c r="F190" s="4"/>
@@ -15230,7 +15234,7 @@
       <c r="O190" s="4"/>
       <c r="P190" s="4"/>
     </row>
-    <row r="191" spans="4:16" x14ac:dyDescent="0.25">
+    <row r="191" spans="4:16" x14ac:dyDescent="0.35">
       <c r="D191" s="4"/>
       <c r="E191" s="4"/>
       <c r="F191" s="4"/>
@@ -15261,9 +15265,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{779F255F-9733-4D52-A7A4-939B0F1BE4F1}">
   <dimension ref="A1:S145"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -15322,7 +15326,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -15381,7 +15385,7 @@
         <v>41.48</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -15440,7 +15444,7 @@
         <v>81.239999999999995</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -15499,7 +15503,7 @@
         <v>115.12</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -15558,7 +15562,7 @@
         <v>150.19999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -15617,7 +15621,7 @@
         <v>186.6</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -15676,7 +15680,7 @@
         <v>223.52</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -15735,7 +15739,7 @@
         <v>259.24</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -15794,7 +15798,7 @@
         <v>293.95999999999998</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -15853,7 +15857,7 @@
         <v>326.88</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -15912,7 +15916,7 @@
         <v>358.32</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -15971,7 +15975,7 @@
         <v>387.28</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -16030,7 +16034,7 @@
         <v>414.24</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -16089,7 +16093,7 @@
         <v>439.84</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -16148,7 +16152,7 @@
         <v>463.68</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -16207,7 +16211,7 @@
         <v>484.96</v>
       </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>13</v>
       </c>
@@ -16266,7 +16270,7 @@
         <v>502.64</v>
       </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>13</v>
       </c>
@@ -16325,7 +16329,7 @@
         <v>517.67999999999995</v>
       </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>13</v>
       </c>
@@ -16384,7 +16388,7 @@
         <v>530.91999999999996</v>
       </c>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>13</v>
       </c>
@@ -16443,7 +16447,7 @@
         <v>542.08000000000004</v>
       </c>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>13</v>
       </c>
@@ -16502,7 +16506,7 @@
         <v>551.04</v>
       </c>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>13</v>
       </c>
@@ -16561,7 +16565,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>13</v>
       </c>
@@ -16620,7 +16624,7 @@
         <v>563.24</v>
       </c>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>13</v>
       </c>
@@ -16679,7 +16683,7 @@
         <v>566.44000000000005</v>
       </c>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>13</v>
       </c>
@@ -16738,7 +16742,7 @@
         <v>568.16</v>
       </c>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>13</v>
       </c>
@@ -16797,7 +16801,7 @@
         <v>530.48</v>
       </c>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>13</v>
       </c>
@@ -16856,7 +16860,7 @@
         <v>493.56</v>
       </c>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>13</v>
       </c>
@@ -16915,7 +16919,7 @@
         <v>461.92</v>
       </c>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>13</v>
       </c>
@@ -16974,7 +16978,7 @@
         <v>430.72</v>
       </c>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>13</v>
       </c>
@@ -17033,7 +17037,7 @@
         <v>400.84</v>
       </c>
     </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>13</v>
       </c>
@@ -17092,7 +17096,7 @@
         <v>368.88</v>
       </c>
     </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>13</v>
       </c>
@@ -17151,7 +17155,7 @@
         <v>336.56</v>
       </c>
     </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>13</v>
       </c>
@@ -17210,7 +17214,7 @@
         <v>304.68</v>
       </c>
     </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>13</v>
       </c>
@@ -17269,7 +17273,7 @@
         <v>276.8</v>
       </c>
     </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>13</v>
       </c>
@@ -17328,7 +17332,7 @@
         <v>249.48</v>
       </c>
     </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>13</v>
       </c>
@@ -17387,7 +17391,7 @@
         <v>223.28</v>
       </c>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>13</v>
       </c>
@@ -17446,7 +17450,7 @@
         <v>198.96</v>
       </c>
     </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>13</v>
       </c>
@@ -17505,7 +17509,7 @@
         <v>175.72</v>
       </c>
     </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>13</v>
       </c>
@@ -17564,7 +17568,7 @@
         <v>152.68</v>
       </c>
     </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>13</v>
       </c>
@@ -17623,7 +17627,7 @@
         <v>131.47999999999999</v>
       </c>
     </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>13</v>
       </c>
@@ -17682,7 +17686,7 @@
         <v>114.4</v>
       </c>
     </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>13</v>
       </c>
@@ -17741,7 +17745,7 @@
         <v>99.96</v>
       </c>
     </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>13</v>
       </c>
@@ -17800,7 +17804,7 @@
         <v>88.24</v>
       </c>
     </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>13</v>
       </c>
@@ -17859,7 +17863,7 @@
         <v>79.52</v>
       </c>
     </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>13</v>
       </c>
@@ -17918,7 +17922,7 @@
         <v>73.239999999999995</v>
       </c>
     </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>13</v>
       </c>
@@ -17977,7 +17981,7 @@
         <v>69.48</v>
       </c>
     </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>13</v>
       </c>
@@ -18036,7 +18040,7 @@
         <v>67.52</v>
       </c>
     </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>13</v>
       </c>
@@ -18095,7 +18099,7 @@
         <v>67.72</v>
       </c>
     </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>13</v>
       </c>
@@ -18154,7 +18158,7 @@
         <v>70.08</v>
       </c>
     </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>13</v>
       </c>
@@ -18213,7 +18217,7 @@
         <v>70.84</v>
       </c>
     </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>13</v>
       </c>
@@ -18272,7 +18276,7 @@
         <v>72.8</v>
       </c>
     </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>13</v>
       </c>
@@ -18331,7 +18335,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>13</v>
       </c>
@@ -18390,7 +18394,7 @@
         <v>75.84</v>
       </c>
     </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>13</v>
       </c>
@@ -18449,7 +18453,7 @@
         <v>74.2</v>
       </c>
     </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>13</v>
       </c>
@@ -18508,7 +18512,7 @@
         <v>74.319999999999993</v>
       </c>
     </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>13</v>
       </c>
@@ -18567,7 +18571,7 @@
         <v>76.319999999999993</v>
       </c>
     </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>13</v>
       </c>
@@ -18626,7 +18630,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>13</v>
       </c>
@@ -18685,7 +18689,7 @@
         <v>78.8</v>
       </c>
     </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>13</v>
       </c>
@@ -18744,7 +18748,7 @@
         <v>79.239999999999995</v>
       </c>
     </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>13</v>
       </c>
@@ -18803,7 +18807,7 @@
         <v>81.12</v>
       </c>
     </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>13</v>
       </c>
@@ -18862,7 +18866,7 @@
         <v>83.12</v>
       </c>
     </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>13</v>
       </c>
@@ -18921,7 +18925,7 @@
         <v>84.96</v>
       </c>
     </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>13</v>
       </c>
@@ -18980,7 +18984,7 @@
         <v>87.8</v>
       </c>
     </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>13</v>
       </c>
@@ -19039,7 +19043,7 @@
         <v>91.4</v>
       </c>
     </row>
-    <row r="65" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>13</v>
       </c>
@@ -19098,7 +19102,7 @@
         <v>94.56</v>
       </c>
     </row>
-    <row r="66" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>13</v>
       </c>
@@ -19157,7 +19161,7 @@
         <v>97.72</v>
       </c>
     </row>
-    <row r="67" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>13</v>
       </c>
@@ -19216,7 +19220,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="68" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>13</v>
       </c>
@@ -19275,7 +19279,7 @@
         <v>101.28</v>
       </c>
     </row>
-    <row r="69" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>13</v>
       </c>
@@ -19334,7 +19338,7 @@
         <v>102.32</v>
       </c>
     </row>
-    <row r="70" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>13</v>
       </c>
@@ -19393,7 +19397,7 @@
         <v>102.48</v>
       </c>
     </row>
-    <row r="71" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>13</v>
       </c>
@@ -19452,7 +19456,7 @@
         <v>102.28</v>
       </c>
     </row>
-    <row r="72" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>13</v>
       </c>
@@ -19511,7 +19515,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="73" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>13</v>
       </c>
@@ -19570,7 +19574,7 @@
         <v>101.08</v>
       </c>
     </row>
-    <row r="74" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>13</v>
       </c>
@@ -19629,7 +19633,7 @@
         <v>99.56</v>
       </c>
     </row>
-    <row r="75" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>13</v>
       </c>
@@ -19688,7 +19692,7 @@
         <v>97.44</v>
       </c>
     </row>
-    <row r="76" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>13</v>
       </c>
@@ -19747,7 +19751,7 @@
         <v>95.64</v>
       </c>
     </row>
-    <row r="77" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>13</v>
       </c>
@@ -19806,7 +19810,7 @@
         <v>93.64</v>
       </c>
     </row>
-    <row r="78" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>13</v>
       </c>
@@ -19865,7 +19869,7 @@
         <v>91.52</v>
       </c>
     </row>
-    <row r="79" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>13</v>
       </c>
@@ -19924,7 +19928,7 @@
         <v>89.32</v>
       </c>
     </row>
-    <row r="80" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>13</v>
       </c>
@@ -19983,7 +19987,7 @@
         <v>86.88</v>
       </c>
     </row>
-    <row r="81" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>13</v>
       </c>
@@ -20042,7 +20046,7 @@
         <v>84.4</v>
       </c>
     </row>
-    <row r="82" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>13</v>
       </c>
@@ -20101,7 +20105,7 @@
         <v>82.64</v>
       </c>
     </row>
-    <row r="83" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>13</v>
       </c>
@@ -20160,7 +20164,7 @@
         <v>81.16</v>
       </c>
     </row>
-    <row r="84" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>13</v>
       </c>
@@ -20219,7 +20223,7 @@
         <v>79.599999999999994</v>
       </c>
     </row>
-    <row r="85" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>13</v>
       </c>
@@ -20278,7 +20282,7 @@
         <v>78.040000000000006</v>
       </c>
     </row>
-    <row r="86" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>13</v>
       </c>
@@ -20337,7 +20341,7 @@
         <v>76.92</v>
       </c>
     </row>
-    <row r="87" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>13</v>
       </c>
@@ -20396,7 +20400,7 @@
         <v>76.12</v>
       </c>
     </row>
-    <row r="88" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>13</v>
       </c>
@@ -20455,7 +20459,7 @@
         <v>74.92</v>
       </c>
     </row>
-    <row r="89" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>13</v>
       </c>
@@ -20514,7 +20518,7 @@
         <v>73.599999999999994</v>
       </c>
     </row>
-    <row r="90" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>13</v>
       </c>
@@ -20573,7 +20577,7 @@
         <v>72.28</v>
       </c>
     </row>
-    <row r="91" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>13</v>
       </c>
@@ -20632,7 +20636,7 @@
         <v>70.72</v>
       </c>
     </row>
-    <row r="92" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>13</v>
       </c>
@@ -20691,7 +20695,7 @@
         <v>69.28</v>
       </c>
     </row>
-    <row r="93" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>13</v>
       </c>
@@ -20750,7 +20754,7 @@
         <v>67.88</v>
       </c>
     </row>
-    <row r="94" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>13</v>
       </c>
@@ -20809,7 +20813,7 @@
         <v>66.84</v>
       </c>
     </row>
-    <row r="95" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>13</v>
       </c>
@@ -20868,7 +20872,7 @@
         <v>66.08</v>
       </c>
     </row>
-    <row r="96" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>13</v>
       </c>
@@ -20927,7 +20931,7 @@
         <v>65.36</v>
       </c>
     </row>
-    <row r="97" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>13</v>
       </c>
@@ -20986,7 +20990,7 @@
         <v>64.64</v>
       </c>
     </row>
-    <row r="98" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>13</v>
       </c>
@@ -21045,7 +21049,7 @@
         <v>64.040000000000006</v>
       </c>
     </row>
-    <row r="99" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>13</v>
       </c>
@@ -21104,7 +21108,7 @@
         <v>63.8</v>
       </c>
     </row>
-    <row r="100" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>13</v>
       </c>
@@ -21163,7 +21167,7 @@
         <v>63.56</v>
       </c>
     </row>
-    <row r="101" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>13</v>
       </c>
@@ -21222,7 +21226,7 @@
         <v>63.28</v>
       </c>
     </row>
-    <row r="102" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>13</v>
       </c>
@@ -21281,7 +21285,7 @@
         <v>62.96</v>
       </c>
     </row>
-    <row r="103" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>13</v>
       </c>
@@ -21340,7 +21344,7 @@
         <v>62.52</v>
       </c>
     </row>
-    <row r="104" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>13</v>
       </c>
@@ -21399,7 +21403,7 @@
         <v>62.04</v>
       </c>
     </row>
-    <row r="105" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>13</v>
       </c>
@@ -21458,7 +21462,7 @@
         <v>61.4</v>
       </c>
     </row>
-    <row r="106" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>13</v>
       </c>
@@ -21517,7 +21521,7 @@
         <v>60.48</v>
       </c>
     </row>
-    <row r="107" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>13</v>
       </c>
@@ -21576,7 +21580,7 @@
         <v>59.52</v>
       </c>
     </row>
-    <row r="108" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>13</v>
       </c>
@@ -21635,7 +21639,7 @@
         <v>58.56</v>
       </c>
     </row>
-    <row r="109" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>13</v>
       </c>
@@ -21694,7 +21698,7 @@
         <v>57.64</v>
       </c>
     </row>
-    <row r="110" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>13</v>
       </c>
@@ -21753,7 +21757,7 @@
         <v>56.6</v>
       </c>
     </row>
-    <row r="111" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>13</v>
       </c>
@@ -21812,7 +21816,7 @@
         <v>55.76</v>
       </c>
     </row>
-    <row r="112" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>13</v>
       </c>
@@ -21871,7 +21875,7 @@
         <v>55.28</v>
       </c>
     </row>
-    <row r="113" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>13</v>
       </c>
@@ -21930,7 +21934,7 @@
         <v>54.88</v>
       </c>
     </row>
-    <row r="114" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>13</v>
       </c>
@@ -21989,7 +21993,7 @@
         <v>54.52</v>
       </c>
     </row>
-    <row r="115" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>13</v>
       </c>
@@ -22048,7 +22052,7 @@
         <v>54.36</v>
       </c>
     </row>
-    <row r="116" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>13</v>
       </c>
@@ -22107,7 +22111,7 @@
         <v>54.16</v>
       </c>
     </row>
-    <row r="117" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>13</v>
       </c>
@@ -22166,7 +22170,7 @@
         <v>53.92</v>
       </c>
     </row>
-    <row r="118" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>13</v>
       </c>
@@ -22225,7 +22229,7 @@
         <v>53.64</v>
       </c>
     </row>
-    <row r="119" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>13</v>
       </c>
@@ -22284,7 +22288,7 @@
         <v>53.36</v>
       </c>
     </row>
-    <row r="120" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>13</v>
       </c>
@@ -22343,7 +22347,7 @@
         <v>53.04</v>
       </c>
     </row>
-    <row r="121" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>13</v>
       </c>
@@ -22402,7 +22406,7 @@
         <v>52.68</v>
       </c>
     </row>
-    <row r="122" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>13</v>
       </c>
@@ -22461,7 +22465,7 @@
         <v>52.4</v>
       </c>
     </row>
-    <row r="123" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>13</v>
       </c>
@@ -22520,7 +22524,7 @@
         <v>52.12</v>
       </c>
     </row>
-    <row r="124" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>13</v>
       </c>
@@ -22579,7 +22583,7 @@
         <v>51.76</v>
       </c>
     </row>
-    <row r="125" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>13</v>
       </c>
@@ -22638,7 +22642,7 @@
         <v>51.32</v>
       </c>
     </row>
-    <row r="126" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>13</v>
       </c>
@@ -22697,7 +22701,7 @@
         <v>50.92</v>
       </c>
     </row>
-    <row r="127" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>13</v>
       </c>
@@ -22756,7 +22760,7 @@
         <v>50.52</v>
       </c>
     </row>
-    <row r="128" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>13</v>
       </c>
@@ -22815,7 +22819,7 @@
         <v>50.04</v>
       </c>
     </row>
-    <row r="129" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>13</v>
       </c>
@@ -22874,7 +22878,7 @@
         <v>49.56</v>
       </c>
     </row>
-    <row r="130" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>13</v>
       </c>
@@ -22933,7 +22937,7 @@
         <v>49.36</v>
       </c>
     </row>
-    <row r="131" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>13</v>
       </c>
@@ -22992,7 +22996,7 @@
         <v>49.2</v>
       </c>
     </row>
-    <row r="132" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>13</v>
       </c>
@@ -23051,7 +23055,7 @@
         <v>49.04</v>
       </c>
     </row>
-    <row r="133" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>13</v>
       </c>
@@ -23110,7 +23114,7 @@
         <v>48.84</v>
       </c>
     </row>
-    <row r="134" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>13</v>
       </c>
@@ -23169,7 +23173,7 @@
         <v>48.72</v>
       </c>
     </row>
-    <row r="135" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>13</v>
       </c>
@@ -23228,7 +23232,7 @@
         <v>48.64</v>
       </c>
     </row>
-    <row r="136" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>13</v>
       </c>
@@ -23287,7 +23291,7 @@
         <v>48.52</v>
       </c>
     </row>
-    <row r="137" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>13</v>
       </c>
@@ -23346,7 +23350,7 @@
         <v>48.32</v>
       </c>
     </row>
-    <row r="138" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>13</v>
       </c>
@@ -23405,7 +23409,7 @@
         <v>48.08</v>
       </c>
     </row>
-    <row r="139" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>13</v>
       </c>
@@ -23464,7 +23468,7 @@
         <v>47.88</v>
       </c>
     </row>
-    <row r="140" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>13</v>
       </c>
@@ -23523,7 +23527,7 @@
         <v>47.72</v>
       </c>
     </row>
-    <row r="141" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>13</v>
       </c>
@@ -23582,7 +23586,7 @@
         <v>47.56</v>
       </c>
     </row>
-    <row r="142" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>13</v>
       </c>
@@ -23641,7 +23645,7 @@
         <v>47.44</v>
       </c>
     </row>
-    <row r="143" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>13</v>
       </c>
@@ -23700,7 +23704,7 @@
         <v>47.16</v>
       </c>
     </row>
-    <row r="144" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>13</v>
       </c>
@@ -23759,7 +23763,7 @@
         <v>46.84</v>
       </c>
     </row>
-    <row r="145" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>13</v>
       </c>

</xml_diff>